<commit_message>
feat: build unified ai test design input
</commit_message>
<xml_diff>
--- a/.example/.tirai/outputs/excel/test-cases.xlsx
+++ b/.example/.tirai/outputs/excel/test-cases.xlsx
@@ -4,18 +4,44 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Test Cases" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Steps" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Expected Results" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Data Needs" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Summary" state="visible" r:id="rId8"/>
+    <sheet sheetId="1" name="Contract Summary" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Test Cases" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="UI Checks" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="API Checks" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="State Checks" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Traceability" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Steps" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Expected Results" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Data Needs" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Summary" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="176">
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Contract Fingerprint</t>
+  </si>
+  <si>
+    <t>3a1f964edd3648be2c80947fa190e11f9f2352f71d42eb86a33c71eeacd3e843</t>
+  </si>
+  <si>
+    <t>Contract Version</t>
+  </si>
+  <si>
+    <t>Test Plan Fingerprint</t>
+  </si>
+  <si>
+    <t>50921188dde047f0b371c434714535e4d06639e3ae84fbb99f08455a44bb3152</t>
+  </si>
   <si>
     <t>ID</t>
   </si>
@@ -38,6 +64,18 @@
     <t>Requirement IDs</t>
   </si>
   <si>
+    <t>Preconditions</t>
+  </si>
+  <si>
+    <t>Test Data</t>
+  </si>
+  <si>
+    <t>Cleanup</t>
+  </si>
+  <si>
+    <t>Automation Reason</t>
+  </si>
+  <si>
     <t>TC-BF-001</t>
   </si>
   <si>
@@ -59,6 +97,9 @@
     <t>REQ-BF-001</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>TC-BF-002</t>
   </si>
   <si>
@@ -122,6 +163,9 @@
     <t>REQ-BF-006</t>
   </si>
   <si>
+    <t>Requires a trusted API fixture and optimistic-cache assertion for the created row.</t>
+  </si>
+  <si>
     <t>TC-BF-007</t>
   </si>
   <si>
@@ -149,6 +193,9 @@
     <t>REQ-BF-008</t>
   </si>
   <si>
+    <t>Requires a stable row identity or API fixture binding for the dynamic todo list.</t>
+  </si>
+  <si>
     <t>TC-BF-009</t>
   </si>
   <si>
@@ -233,6 +280,9 @@
     <t>REQ-BF-015</t>
   </si>
   <si>
+    <t>Requires a stable user-row action locator or API fixture binding.</t>
+  </si>
+  <si>
     <t>TC-BF-016</t>
   </si>
   <si>
@@ -245,6 +295,9 @@
     <t>REQ-BF-016</t>
   </si>
   <si>
+    <t>Requires a stable user-row action locator and dialog fixture.</t>
+  </si>
+  <si>
     <t>TC-BF-017</t>
   </si>
   <si>
@@ -257,18 +310,195 @@
     <t>REQ-BF-017</t>
   </si>
   <si>
+    <t>Requires a stable user-row action locator and trusted PATCH fixture.</t>
+  </si>
+  <si>
     <t>TestCase ID</t>
   </si>
   <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>The browser title is TanStack Full Demo.</t>
+  </si>
+  <si>
+    <t>TanStack Full Demo</t>
+  </si>
+  <si>
+    <t>The dashboard heading is visible.</t>
+  </si>
+  <si>
+    <t>dashboard-heading</t>
+  </si>
+  <si>
+    <t>The browser navigates to the Todos route.</t>
+  </si>
+  <si>
+    <t>/todos</t>
+  </si>
+  <si>
+    <t>The Todos page heading is visible.</t>
+  </si>
+  <si>
+    <t>todos-heading</t>
+  </si>
+  <si>
+    <t>The title validation message is shown.</t>
+  </si>
+  <si>
+    <t>add-todo-validation</t>
+  </si>
+  <si>
+    <t>Title is required</t>
+  </si>
+  <si>
+    <t>The Add Todo form remains available after submit.</t>
+  </si>
+  <si>
+    <t>add-todo-input</t>
+  </si>
+  <si>
+    <t>The search control contains the entered query.</t>
+  </si>
+  <si>
+    <t>todo-search</t>
+  </si>
+  <si>
+    <t>buy milk</t>
+  </si>
+  <si>
+    <t>A Todo row is available for status transition.</t>
+  </si>
+  <si>
+    <t>todo-row</t>
+  </si>
+  <si>
+    <t>A Todo row is available for deletion.</t>
+  </si>
+  <si>
+    <t>The Posts page heading is visible.</t>
+  </si>
+  <si>
+    <t>posts-heading</t>
+  </si>
+  <si>
+    <t>The Posts filter contains the entered query.</t>
+  </si>
+  <si>
+    <t>posts-filter</t>
+  </si>
+  <si>
+    <t>tanstack</t>
+  </si>
+  <si>
+    <t>The virtual-list view control remains enabled.</t>
+  </si>
+  <si>
+    <t>posts-virtual-view</t>
+  </si>
+  <si>
+    <t>The Users page heading is visible.</t>
+  </si>
+  <si>
+    <t>users-heading</t>
+  </si>
+  <si>
+    <t>The Users filter contains the entered query.</t>
+  </si>
+  <si>
+    <t>users-filter</t>
+  </si>
+  <si>
+    <t>Leanne</t>
+  </si>
+  <si>
+    <t>A user row is available for editing.</t>
+  </si>
+  <si>
+    <t>user-row</t>
+  </si>
+  <si>
+    <t>The edit dialog form is available for validation.</t>
+  </si>
+  <si>
+    <t>edit-user-dialog</t>
+  </si>
+  <si>
+    <t>The Users page remains available for update.</t>
+  </si>
+  <si>
+    <t>Scenario ID</t>
+  </si>
+  <si>
+    <t>Provenance</t>
+  </si>
+  <si>
+    <t>SC-BF-001</t>
+  </si>
+  <si>
+    <t>ctx-72bf0e82f91621cacf990d81</t>
+  </si>
+  <si>
+    <t>SC-BF-002</t>
+  </si>
+  <si>
+    <t>SC-BF-003</t>
+  </si>
+  <si>
+    <t>SC-BF-004</t>
+  </si>
+  <si>
+    <t>SC-BF-005</t>
+  </si>
+  <si>
+    <t>SC-BF-006</t>
+  </si>
+  <si>
+    <t>SC-BF-007</t>
+  </si>
+  <si>
+    <t>SC-BF-008</t>
+  </si>
+  <si>
+    <t>SC-BF-009</t>
+  </si>
+  <si>
+    <t>SC-BF-010</t>
+  </si>
+  <si>
+    <t>SC-BF-011</t>
+  </si>
+  <si>
+    <t>SC-BF-012</t>
+  </si>
+  <si>
+    <t>SC-BF-013</t>
+  </si>
+  <si>
+    <t>SC-BF-014</t>
+  </si>
+  <si>
+    <t>SC-BF-015</t>
+  </si>
+  <si>
+    <t>SC-BF-016</t>
+  </si>
+  <si>
+    <t>SC-BF-017</t>
+  </si>
+  <si>
     <t>Order</t>
   </si>
   <si>
     <t>Action</t>
   </si>
   <si>
-    <t>Target</t>
-  </si>
-  <si>
     <t>navigate</t>
   </si>
   <si>
@@ -281,100 +511,25 @@
     <t>nav-todos</t>
   </si>
   <si>
-    <t>/todos</t>
-  </si>
-  <si>
     <t>fill</t>
   </si>
   <si>
-    <t>add-todo-input</t>
-  </si>
-  <si>
     <t>blur</t>
   </si>
   <si>
     <t>add-todo-button</t>
   </si>
   <si>
-    <t>todo-search</t>
-  </si>
-  <si>
     <t>/posts</t>
   </si>
   <si>
-    <t>posts-filter</t>
-  </si>
-  <si>
-    <t>posts-virtual-view</t>
-  </si>
-  <si>
     <t>/users</t>
   </si>
   <si>
-    <t>users-filter</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Verification Type</t>
   </si>
   <si>
-    <t>The browser title is TanStack Full Demo.</t>
-  </si>
-  <si>
-    <t>The dashboard heading is visible.</t>
-  </si>
-  <si>
-    <t>The browser navigates to the Todos route.</t>
-  </si>
-  <si>
-    <t>The Todos page heading is visible.</t>
-  </si>
-  <si>
-    <t>The title validation message is shown.</t>
-  </si>
-  <si>
-    <t>The Add Todo form remains available after submit.</t>
-  </si>
-  <si>
-    <t>The search control contains the entered query.</t>
-  </si>
-  <si>
-    <t>A Todo row is available for status transition.</t>
-  </si>
-  <si>
-    <t>A Todo row is available for deletion.</t>
-  </si>
-  <si>
-    <t>The Posts page heading is visible.</t>
-  </si>
-  <si>
-    <t>The Posts filter contains the entered query.</t>
-  </si>
-  <si>
-    <t>The virtual-list view control remains enabled.</t>
-  </si>
-  <si>
-    <t>The Users page heading is visible.</t>
-  </si>
-  <si>
-    <t>The Users filter contains the entered query.</t>
-  </si>
-  <si>
-    <t>A user row is available for editing.</t>
-  </si>
-  <si>
-    <t>The edit dialog form is available for validation.</t>
-  </si>
-  <si>
-    <t>The Users page remains available for update.</t>
-  </si>
-  <si>
     <t>Metric</t>
-  </si>
-  <si>
-    <t>Value</t>
   </si>
   <si>
     <t>Total Test Cases</t>
@@ -769,7 +924,117 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -778,420 +1043,639 @@
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="25" customWidth="1"/>
+    <col min="8" max="9" width="45" customWidth="1"/>
+    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="11" max="11" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="H2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" t="s">
+      <c r="F5" t="s">
         <v>23</v>
       </c>
-      <c r="C5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
       <c r="G5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="H6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="H8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="H9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" t="s">
+        <v>25</v>
+      </c>
+      <c r="K9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
         <v>45</v>
       </c>
-      <c r="C10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" t="s">
-        <v>33</v>
-      </c>
       <c r="G10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="H10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" t="s">
+        <v>25</v>
+      </c>
+      <c r="J10" t="s">
+        <v>25</v>
+      </c>
+      <c r="K10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11" t="s">
+        <v>25</v>
+      </c>
+      <c r="J11" t="s">
+        <v>25</v>
+      </c>
+      <c r="K11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s">
-        <v>38</v>
-      </c>
       <c r="F12" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="H12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12" t="s">
+        <v>25</v>
+      </c>
+      <c r="J12" t="s">
+        <v>25</v>
+      </c>
+      <c r="K12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="H13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="D14" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F14" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+      <c r="H14" t="s">
+        <v>25</v>
+      </c>
+      <c r="I14" t="s">
+        <v>25</v>
+      </c>
+      <c r="J14" t="s">
+        <v>25</v>
+      </c>
+      <c r="K14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="D15" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F15" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="H15" t="s">
+        <v>25</v>
+      </c>
+      <c r="I15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>25</v>
+      </c>
+      <c r="K15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D16" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E16" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F16" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="H16" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16" t="s">
+        <v>25</v>
+      </c>
+      <c r="J16" t="s">
+        <v>25</v>
+      </c>
+      <c r="K16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F17" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="G17" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="H17" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17" t="s">
+        <v>25</v>
+      </c>
+      <c r="J17" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="D18" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F18" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="G18" t="s">
-        <v>79</v>
+        <v>95</v>
+      </c>
+      <c r="H18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K18" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1200,7 +1684,607 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="65" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>122</v>
+      </c>
+      <c r="C12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" t="s">
+        <v>126</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" t="s">
+        <v>127</v>
+      </c>
+      <c r="C14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C15" t="s">
+        <v>130</v>
+      </c>
+      <c r="D15" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" t="s">
+        <v>133</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" t="s">
+        <v>135</v>
+      </c>
+      <c r="D17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="65" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="65" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D9" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>149</v>
+      </c>
+      <c r="D11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D12" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" t="s">
+        <v>151</v>
+      </c>
+      <c r="D13" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" t="s">
+        <v>152</v>
+      </c>
+      <c r="D14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" t="s">
+        <v>153</v>
+      </c>
+      <c r="D15" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" t="s">
+        <v>154</v>
+      </c>
+      <c r="D16" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" t="s">
+        <v>155</v>
+      </c>
+      <c r="D17" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" t="s">
+        <v>156</v>
+      </c>
+      <c r="D18" t="s">
+        <v>140</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1213,394 +2297,394 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B1" t="s">
-        <v>81</v>
+        <v>157</v>
       </c>
       <c r="C1" t="s">
-        <v>82</v>
+        <v>158</v>
       </c>
       <c r="D1" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D3" t="s">
-        <v>85</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>161</v>
       </c>
       <c r="D5" t="s">
-        <v>87</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D6" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>163</v>
       </c>
       <c r="D8" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>164</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>86</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>92</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D11" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>163</v>
       </c>
       <c r="D12" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B13">
         <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>161</v>
       </c>
       <c r="D13" t="s">
-        <v>92</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>163</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="B17">
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D17" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D18" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D19" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B20">
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>163</v>
       </c>
       <c r="D20" t="s">
-        <v>95</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D21" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B22">
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>86</v>
+        <v>161</v>
       </c>
       <c r="D22" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D23" t="s">
-        <v>97</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D24" t="s">
-        <v>97</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B25">
         <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>163</v>
       </c>
       <c r="D25" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D26" t="s">
-        <v>97</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>167</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>84</v>
+        <v>159</v>
       </c>
       <c r="D28" t="s">
-        <v>97</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -1609,7 +2693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1621,200 +2705,200 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C1" t="s">
-        <v>100</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
         <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="B18" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="C18" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1823,7 +2907,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1835,76 +2919,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B2">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>125</v>
-      </c>
-      <c r="B6">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>